<commit_message>
update admincontroller authcontroller authfinancecontroller invoice invoicecontroller invoiceservice financedto exception
</commit_message>
<xml_diff>
--- a/invoices.xlsx
+++ b/invoices.xlsx
@@ -8,11 +8,14 @@
   <sheets>
     <sheet name="Invoices" r:id="rId3" sheetId="1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Invoices!$A$1:$Z$1</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="79">
   <si>
     <t>id</t>
   </si>
@@ -228,14 +231,38 @@
   </si>
   <si>
     <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>INV005</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>INV006</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="dd-MM-yyyy"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -243,16 +270,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="darkGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="48"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="48"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -260,126 +302,156 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Z9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="2.41796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="8.93359375"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="2.9296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.9765625"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="10.13671875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="7.41015625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.72265625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="7.04296875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="8.25"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="10.11328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="7.59375"/>
     <col min="7" max="7" bestFit="true" customWidth="true" width="11.35546875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="11.265625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.00390625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="15.5390625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.56640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="10.046875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="15.33203125"/>
     <col min="11" max="11" bestFit="true" customWidth="true" width="22.05859375"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="7.4296875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="9.921875"/>
     <col min="13" max="13" bestFit="true" customWidth="true" width="10.13671875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="8.609375"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="12.26171875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.3203125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="8.7578125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="13.671875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="11.51171875"/>
     <col min="17" max="17" bestFit="true" customWidth="true" width="3.76171875"/>
     <col min="18" max="18" bestFit="true" customWidth="true" width="4.9296875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="9.625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="10.75"/>
     <col min="20" max="20" bestFit="true" customWidth="true" width="16.84375"/>
     <col min="21" max="21" bestFit="true" customWidth="true" width="24.30078125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="9.62109375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="10.75"/>
     <col min="23" max="23" bestFit="true" customWidth="true" width="16.9296875"/>
     <col min="24" max="24" bestFit="true" customWidth="true" width="9.34375"/>
     <col min="25" max="25" bestFit="true" customWidth="true" width="11.80078125"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="11.2421875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="11.73046875"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s" s="7">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s" s="7">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s" s="7">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s" s="7">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s" s="7">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s" s="7">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s" s="7">
         <v>6</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s" s="7">
         <v>7</v>
       </c>
-      <c r="I1" t="s" s="0">
+      <c r="I1" t="s" s="7">
         <v>8</v>
       </c>
-      <c r="J1" t="s" s="0">
+      <c r="J1" t="s" s="7">
         <v>9</v>
       </c>
-      <c r="K1" t="s" s="0">
+      <c r="K1" t="s" s="7">
         <v>10</v>
       </c>
-      <c r="L1" t="s" s="0">
+      <c r="L1" t="s" s="7">
         <v>11</v>
       </c>
-      <c r="M1" t="s" s="0">
+      <c r="M1" t="s" s="7">
         <v>12</v>
       </c>
-      <c r="N1" t="s" s="0">
+      <c r="N1" t="s" s="7">
         <v>13</v>
       </c>
-      <c r="O1" t="s" s="0">
+      <c r="O1" t="s" s="7">
         <v>14</v>
       </c>
-      <c r="P1" t="s" s="0">
+      <c r="P1" t="s" s="7">
         <v>15</v>
       </c>
-      <c r="Q1" t="s" s="0">
+      <c r="Q1" t="s" s="7">
         <v>16</v>
       </c>
-      <c r="R1" t="s" s="0">
+      <c r="R1" t="s" s="7">
         <v>17</v>
       </c>
-      <c r="S1" t="s" s="0">
+      <c r="S1" t="s" s="7">
         <v>18</v>
       </c>
-      <c r="T1" t="s" s="0">
+      <c r="T1" t="s" s="7">
         <v>19</v>
       </c>
-      <c r="U1" t="s" s="0">
+      <c r="U1" t="s" s="7">
         <v>20</v>
       </c>
-      <c r="V1" t="s" s="0">
+      <c r="V1" t="s" s="7">
         <v>21</v>
       </c>
-      <c r="W1" t="s" s="0">
+      <c r="W1" t="s" s="7">
         <v>22</v>
       </c>
-      <c r="X1" t="s" s="0">
+      <c r="X1" t="s" s="7">
         <v>23</v>
       </c>
-      <c r="Y1" t="s" s="0">
+      <c r="Y1" t="s" s="7">
         <v>24</v>
       </c>
-      <c r="Z1" t="s" s="0">
+      <c r="Z1" t="s" s="7">
         <v>25</v>
       </c>
     </row>
@@ -623,7 +695,408 @@
         <v>49</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="K5" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="L5" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="M5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="N5" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="O5" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="P5" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="Q5" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="R5" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="S5" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="T5" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="U5" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="V5" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="W5" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="X5" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="Y5" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="Z5" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="J6" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="K6" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="L6" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="M6" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="N6" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="O6" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="P6" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="Q6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="R6" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="S6" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="T6" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="U6" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="V6" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="W6" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="X6" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="Y6" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="Z6" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="1">
+        <v>74</v>
+      </c>
+      <c r="B7" t="s" s="1">
+        <v>75</v>
+      </c>
+      <c r="C7" t="n" s="3">
+        <v>46104.0</v>
+      </c>
+      <c r="D7" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G7" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H7" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="I7" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="J7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="K7" t="s" s="1">
+        <v>36</v>
+      </c>
+      <c r="L7" t="n" s="2">
+        <v>50000.0</v>
+      </c>
+      <c r="M7" t="n" s="3">
+        <v>46023.0</v>
+      </c>
+      <c r="N7" t="s" s="1">
+        <v>39</v>
+      </c>
+      <c r="O7" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="P7" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="Q7" t="s" s="1">
+        <v>41</v>
+      </c>
+      <c r="R7" t="s" s="1">
+        <v>42</v>
+      </c>
+      <c r="S7" t="n" s="2">
+        <v>60000.0</v>
+      </c>
+      <c r="T7" t="s" s="1">
+        <v>44</v>
+      </c>
+      <c r="U7" t="s" s="1">
+        <v>45</v>
+      </c>
+      <c r="V7" t="s" s="1">
+        <v>46</v>
+      </c>
+      <c r="W7" t="s" s="1">
+        <v>47</v>
+      </c>
+      <c r="X7" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="Y7" t="s" s="1">
+        <v>48</v>
+      </c>
+      <c r="Z7" t="s" s="1">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="4">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s" s="4">
+        <v>75</v>
+      </c>
+      <c r="C8" t="n" s="6">
+        <v>46104.0</v>
+      </c>
+      <c r="D8" t="s" s="4">
+        <v>29</v>
+      </c>
+      <c r="E8" t="s" s="4">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s" s="4">
+        <v>31</v>
+      </c>
+      <c r="G8" t="s" s="4">
+        <v>32</v>
+      </c>
+      <c r="H8" t="s" s="4">
+        <v>33</v>
+      </c>
+      <c r="I8" t="s" s="4">
+        <v>34</v>
+      </c>
+      <c r="J8" t="s" s="4">
+        <v>35</v>
+      </c>
+      <c r="K8" t="s" s="4">
+        <v>36</v>
+      </c>
+      <c r="L8" t="n" s="5">
+        <v>50000.0</v>
+      </c>
+      <c r="M8" t="n" s="6">
+        <v>46023.0</v>
+      </c>
+      <c r="N8" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="O8" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="P8" t="s" s="4">
+        <v>30</v>
+      </c>
+      <c r="Q8" t="s" s="4">
+        <v>41</v>
+      </c>
+      <c r="R8" t="s" s="4">
+        <v>42</v>
+      </c>
+      <c r="S8" t="n" s="5">
+        <v>60000.0</v>
+      </c>
+      <c r="T8" t="s" s="4">
+        <v>44</v>
+      </c>
+      <c r="U8" t="s" s="4">
+        <v>45</v>
+      </c>
+      <c r="V8" t="s" s="4">
+        <v>46</v>
+      </c>
+      <c r="W8" t="s" s="4">
+        <v>47</v>
+      </c>
+      <c r="X8" t="s" s="4">
+        <v>33</v>
+      </c>
+      <c r="Y8" t="s" s="4">
+        <v>48</v>
+      </c>
+      <c r="Z8" t="s" s="4">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="8">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s" s="8">
+        <v>78</v>
+      </c>
+      <c r="C9" t="n" s="10">
+        <v>46104.0</v>
+      </c>
+      <c r="D9" t="s" s="8">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s" s="8">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s" s="8">
+        <v>31</v>
+      </c>
+      <c r="G9" t="s" s="8">
+        <v>32</v>
+      </c>
+      <c r="H9" t="s" s="8">
+        <v>33</v>
+      </c>
+      <c r="I9" t="s" s="8">
+        <v>34</v>
+      </c>
+      <c r="J9" t="s" s="8">
+        <v>35</v>
+      </c>
+      <c r="K9" t="s" s="8">
+        <v>36</v>
+      </c>
+      <c r="L9" t="n" s="9">
+        <v>50000.0</v>
+      </c>
+      <c r="M9" t="n" s="10">
+        <v>46023.0</v>
+      </c>
+      <c r="N9" t="s" s="8">
+        <v>39</v>
+      </c>
+      <c r="O9" t="s" s="8">
+        <v>40</v>
+      </c>
+      <c r="P9" t="s" s="8">
+        <v>30</v>
+      </c>
+      <c r="Q9" t="s" s="8">
+        <v>41</v>
+      </c>
+      <c r="R9" t="s" s="8">
+        <v>42</v>
+      </c>
+      <c r="S9" t="n" s="9">
+        <v>60000.0</v>
+      </c>
+      <c r="T9" t="s" s="8">
+        <v>44</v>
+      </c>
+      <c r="U9" t="s" s="8">
+        <v>45</v>
+      </c>
+      <c r="V9" t="s" s="8">
+        <v>46</v>
+      </c>
+      <c r="W9" t="s" s="8">
+        <v>47</v>
+      </c>
+      <c r="X9" t="s" s="8">
+        <v>33</v>
+      </c>
+      <c r="Y9" t="s" s="8">
+        <v>48</v>
+      </c>
+      <c r="Z9" t="s" s="8">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:Z1"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated invoiceservice and incvoices.xlsx
</commit_message>
<xml_diff>
--- a/invoices.xlsx
+++ b/invoices.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="51">
   <si>
     <t>S.No</t>
   </si>
@@ -98,13 +98,7 @@
     <t>panNumber</t>
   </si>
   <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>21</t>
+    <t>1</t>
   </si>
   <si>
     <t>INV001</t>
@@ -164,13 +158,16 @@
     <t>AAECT2610C</t>
   </si>
   <si>
-    <t>22</t>
+    <t>2</t>
   </si>
   <si>
     <t>INV002</t>
   </si>
   <si>
-    <t>23</t>
+    <t>Client B</t>
+  </si>
+  <si>
+    <t>React Developer</t>
   </si>
 </sst>
 </file>
@@ -181,28 +178,13 @@
     <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
     <numFmt numFmtId="165" formatCode="dd-MM-yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="4">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="12.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="12.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="12.0"/>
-      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -258,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center"/>
@@ -269,22 +251,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
@@ -296,11 +263,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="5.19921875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="2.9296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="2.71484375"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="9.9765625"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="10.13671875"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="8.25"/>
@@ -309,7 +276,7 @@
     <col min="8" max="8" bestFit="true" customWidth="true" width="11.35546875"/>
     <col min="9" max="9" bestFit="true" customWidth="true" width="12.56640625"/>
     <col min="10" max="10" bestFit="true" customWidth="true" width="10.046875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="13.0546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="14.13671875"/>
     <col min="12" max="12" bestFit="true" customWidth="true" width="19.03515625"/>
     <col min="13" max="13" bestFit="true" customWidth="true" width="9.921875"/>
     <col min="14" max="14" bestFit="true" customWidth="true" width="10.13671875"/>
@@ -329,85 +296,85 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="15">
+      <c r="A1" t="s" s="6">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="15">
+      <c r="B1" t="s" s="6">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="15">
+      <c r="C1" t="s" s="6">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="15">
+      <c r="D1" t="s" s="6">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="15">
+      <c r="E1" t="s" s="6">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="15">
+      <c r="F1" t="s" s="6">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="15">
+      <c r="G1" t="s" s="6">
         <v>6</v>
       </c>
-      <c r="H1" t="s" s="15">
+      <c r="H1" t="s" s="6">
         <v>7</v>
       </c>
-      <c r="I1" t="s" s="15">
+      <c r="I1" t="s" s="6">
         <v>8</v>
       </c>
-      <c r="J1" t="s" s="15">
+      <c r="J1" t="s" s="6">
         <v>9</v>
       </c>
-      <c r="K1" t="s" s="15">
+      <c r="K1" t="s" s="6">
         <v>10</v>
       </c>
-      <c r="L1" t="s" s="15">
+      <c r="L1" t="s" s="6">
         <v>11</v>
       </c>
-      <c r="M1" t="s" s="15">
+      <c r="M1" t="s" s="6">
         <v>12</v>
       </c>
-      <c r="N1" t="s" s="15">
+      <c r="N1" t="s" s="6">
         <v>13</v>
       </c>
-      <c r="O1" t="s" s="15">
+      <c r="O1" t="s" s="6">
         <v>14</v>
       </c>
-      <c r="P1" t="s" s="15">
+      <c r="P1" t="s" s="6">
         <v>15</v>
       </c>
-      <c r="Q1" t="s" s="15">
+      <c r="Q1" t="s" s="6">
         <v>16</v>
       </c>
-      <c r="R1" t="s" s="15">
+      <c r="R1" t="s" s="6">
         <v>17</v>
       </c>
-      <c r="S1" t="s" s="15">
+      <c r="S1" t="s" s="6">
         <v>18</v>
       </c>
-      <c r="T1" t="s" s="15">
+      <c r="T1" t="s" s="6">
         <v>19</v>
       </c>
-      <c r="U1" t="s" s="15">
+      <c r="U1" t="s" s="6">
         <v>20</v>
       </c>
-      <c r="V1" t="s" s="15">
+      <c r="V1" t="s" s="6">
         <v>21</v>
       </c>
-      <c r="W1" t="s" s="15">
+      <c r="W1" t="s" s="6">
         <v>22</v>
       </c>
-      <c r="X1" t="s" s="15">
+      <c r="X1" t="s" s="6">
         <v>23</v>
       </c>
-      <c r="Y1" t="s" s="15">
+      <c r="Y1" t="s" s="6">
         <v>24</v>
       </c>
-      <c r="Z1" t="s" s="15">
+      <c r="Z1" t="s" s="6">
         <v>25</v>
       </c>
-      <c r="AA1" t="s" s="15">
+      <c r="AA1" t="s" s="6">
         <v>26</v>
       </c>
     </row>
@@ -421,326 +388,160 @@
       <c r="C2" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="D2" t="s" s="2">
-        <v>28</v>
+      <c r="D2" t="n" s="4">
+        <v>46104.0</v>
       </c>
       <c r="E2" t="s" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H2" t="s" s="2">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="I2" t="s" s="2">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="J2" t="s" s="2">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="K2" t="s" s="2">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="L2" t="s" s="2">
-        <v>28</v>
-      </c>
-      <c r="M2" t="s" s="2">
-        <v>28</v>
-      </c>
-      <c r="N2" t="s" s="2">
-        <v>28</v>
+        <v>36</v>
+      </c>
+      <c r="M2" t="n" s="3">
+        <v>50000.0</v>
+      </c>
+      <c r="N2" t="n" s="4">
+        <v>46023.0</v>
       </c>
       <c r="O2" t="s" s="2">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="P2" t="s" s="2">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q2" t="s" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="R2" t="s" s="2">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="S2" t="s" s="2">
-        <v>28</v>
-      </c>
-      <c r="T2" t="s" s="2">
-        <v>28</v>
+        <v>40</v>
+      </c>
+      <c r="T2" t="n" s="3">
+        <v>60000.0</v>
       </c>
       <c r="U2" t="s" s="2">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="V2" t="s" s="2">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="W2" t="s" s="2">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="X2" t="s" s="2">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="Y2" t="s" s="2">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="Z2" t="s" s="2">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="AA2" t="s" s="2">
-        <v>28</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n" s="6">
+      <c r="A3" t="n" s="7">
         <v>2.0</v>
       </c>
-      <c r="B3" t="s" s="6">
-        <v>29</v>
-      </c>
-      <c r="C3" t="s" s="6">
+      <c r="B3" t="s" s="7">
+        <v>47</v>
+      </c>
+      <c r="C3" t="s" s="7">
+        <v>48</v>
+      </c>
+      <c r="D3" t="n" s="9">
+        <v>46104.0</v>
+      </c>
+      <c r="E3" t="s" s="7">
+        <v>49</v>
+      </c>
+      <c r="F3" t="s" s="7">
         <v>30</v>
       </c>
-      <c r="D3" t="n" s="8">
-        <v>46104.0</v>
-      </c>
-      <c r="E3" t="s" s="6">
+      <c r="G3" t="s" s="7">
         <v>31</v>
       </c>
-      <c r="F3" t="s" s="6">
+      <c r="H3" t="s" s="7">
         <v>32</v>
       </c>
-      <c r="G3" t="s" s="6">
+      <c r="I3" t="s" s="7">
         <v>33</v>
       </c>
-      <c r="H3" t="s" s="6">
+      <c r="J3" t="s" s="7">
         <v>34</v>
       </c>
-      <c r="I3" t="s" s="6">
-        <v>35</v>
-      </c>
-      <c r="J3" t="s" s="6">
+      <c r="K3" t="s" s="7">
+        <v>50</v>
+      </c>
+      <c r="L3" t="s" s="7">
         <v>36</v>
       </c>
-      <c r="K3" t="s" s="6">
+      <c r="M3" t="n" s="8">
+        <v>50000.0</v>
+      </c>
+      <c r="N3" t="n" s="9">
+        <v>46023.0</v>
+      </c>
+      <c r="O3" t="s" s="7">
         <v>37</v>
       </c>
-      <c r="L3" t="s" s="6">
+      <c r="P3" t="s" s="7">
         <v>38</v>
       </c>
-      <c r="M3" t="n" s="7">
-        <v>50000.0</v>
-      </c>
-      <c r="N3" t="n" s="8">
-        <v>46023.0</v>
-      </c>
-      <c r="O3" t="s" s="6">
+      <c r="Q3" t="s" s="7">
+        <v>30</v>
+      </c>
+      <c r="R3" t="s" s="7">
         <v>39</v>
       </c>
-      <c r="P3" t="s" s="6">
+      <c r="S3" t="s" s="7">
         <v>40</v>
       </c>
-      <c r="Q3" t="s" s="6">
-        <v>32</v>
-      </c>
-      <c r="R3" t="s" s="6">
+      <c r="T3" t="n" s="8">
+        <v>60000.0</v>
+      </c>
+      <c r="U3" t="s" s="7">
         <v>41</v>
       </c>
-      <c r="S3" t="s" s="6">
+      <c r="V3" t="s" s="7">
         <v>42</v>
       </c>
-      <c r="T3" t="n" s="7">
-        <v>60000.0</v>
-      </c>
-      <c r="U3" t="s" s="6">
+      <c r="W3" t="s" s="7">
         <v>43</v>
       </c>
-      <c r="V3" t="s" s="6">
+      <c r="X3" t="s" s="7">
         <v>44</v>
       </c>
-      <c r="W3" t="s" s="6">
+      <c r="Y3" t="s" s="7">
+        <v>33</v>
+      </c>
+      <c r="Z3" t="s" s="7">
         <v>45</v>
       </c>
-      <c r="X3" t="s" s="6">
+      <c r="AA3" t="s" s="7">
         <v>46</v>
-      </c>
-      <c r="Y3" t="s" s="6">
-        <v>35</v>
-      </c>
-      <c r="Z3" t="s" s="6">
-        <v>47</v>
-      </c>
-      <c r="AA3" t="s" s="6">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="B4" t="s" s="11">
-        <v>49</v>
-      </c>
-      <c r="C4" t="s" s="11">
-        <v>50</v>
-      </c>
-      <c r="D4" t="n" s="13">
-        <v>46104.0</v>
-      </c>
-      <c r="E4" t="s" s="11">
-        <v>31</v>
-      </c>
-      <c r="F4" t="s" s="11">
-        <v>32</v>
-      </c>
-      <c r="G4" t="s" s="11">
-        <v>33</v>
-      </c>
-      <c r="H4" t="s" s="11">
-        <v>34</v>
-      </c>
-      <c r="I4" t="s" s="11">
-        <v>35</v>
-      </c>
-      <c r="J4" t="s" s="11">
-        <v>36</v>
-      </c>
-      <c r="K4" t="s" s="11">
-        <v>37</v>
-      </c>
-      <c r="L4" t="s" s="11">
-        <v>38</v>
-      </c>
-      <c r="M4" t="n" s="12">
-        <v>50000.0</v>
-      </c>
-      <c r="N4" t="n" s="13">
-        <v>46023.0</v>
-      </c>
-      <c r="O4" t="s" s="11">
-        <v>39</v>
-      </c>
-      <c r="P4" t="s" s="11">
-        <v>40</v>
-      </c>
-      <c r="Q4" t="s" s="11">
-        <v>32</v>
-      </c>
-      <c r="R4" t="s" s="11">
-        <v>41</v>
-      </c>
-      <c r="S4" t="s" s="11">
-        <v>42</v>
-      </c>
-      <c r="T4" t="n" s="12">
-        <v>60000.0</v>
-      </c>
-      <c r="U4" t="s" s="11">
-        <v>43</v>
-      </c>
-      <c r="V4" t="s" s="11">
-        <v>44</v>
-      </c>
-      <c r="W4" t="s" s="11">
-        <v>45</v>
-      </c>
-      <c r="X4" t="s" s="11">
-        <v>46</v>
-      </c>
-      <c r="Y4" t="s" s="11">
-        <v>35</v>
-      </c>
-      <c r="Z4" t="s" s="11">
-        <v>47</v>
-      </c>
-      <c r="AA4" t="s" s="11">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="B5" t="s" s="16">
-        <v>51</v>
-      </c>
-      <c r="C5" t="s" s="16">
-        <v>30</v>
-      </c>
-      <c r="D5" t="n" s="18">
-        <v>46104.0</v>
-      </c>
-      <c r="E5" t="s" s="16">
-        <v>31</v>
-      </c>
-      <c r="F5" t="s" s="16">
-        <v>32</v>
-      </c>
-      <c r="G5" t="s" s="16">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s" s="16">
-        <v>34</v>
-      </c>
-      <c r="I5" t="s" s="16">
-        <v>35</v>
-      </c>
-      <c r="J5" t="s" s="16">
-        <v>36</v>
-      </c>
-      <c r="K5" t="s" s="16">
-        <v>37</v>
-      </c>
-      <c r="L5" t="s" s="16">
-        <v>38</v>
-      </c>
-      <c r="M5" t="n" s="17">
-        <v>50000.0</v>
-      </c>
-      <c r="N5" t="n" s="18">
-        <v>46023.0</v>
-      </c>
-      <c r="O5" t="s" s="16">
-        <v>39</v>
-      </c>
-      <c r="P5" t="s" s="16">
-        <v>40</v>
-      </c>
-      <c r="Q5" t="s" s="16">
-        <v>32</v>
-      </c>
-      <c r="R5" t="s" s="16">
-        <v>41</v>
-      </c>
-      <c r="S5" t="s" s="16">
-        <v>42</v>
-      </c>
-      <c r="T5" t="n" s="17">
-        <v>60000.0</v>
-      </c>
-      <c r="U5" t="s" s="16">
-        <v>43</v>
-      </c>
-      <c r="V5" t="s" s="16">
-        <v>44</v>
-      </c>
-      <c r="W5" t="s" s="16">
-        <v>45</v>
-      </c>
-      <c r="X5" t="s" s="16">
-        <v>46</v>
-      </c>
-      <c r="Y5" t="s" s="16">
-        <v>35</v>
-      </c>
-      <c r="Z5" t="s" s="16">
-        <v>47</v>
-      </c>
-      <c r="AA5" t="s" s="16">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>